<commit_message>
test: adding a live search-quality regression suite and expanding the dataset
Grows the sample catalog to 40 pairs across five categories and adds a quality
suite that measures what no unit test can: whether a person's own phrasing finds
the right pair, and whether a question the catalog cannot answer is correctly
refused rather than answered from an unrelated pair. The refusal half is the one
that decays silently — a retriever that answers everything passes every other
test and quietly empties the gap report.

Marked `quality` and deselected by default, since it needs a live deployment
with real embeddings; it points at the /api/v1 endpoints and skips cleanly when
no stack is reachable.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TtXzgtguxDEByQy9dSHcoh
</commit_message>
<xml_diff>
--- a/examples/qa_catalog_sample.xlsx
+++ b/examples/qa_catalog_sample.xlsx
@@ -7,14 +7,14 @@
     <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
   </bookViews>
   <sheets>
-    <sheet name="qa_pairs" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="82">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="165" uniqueCount="130">
   <si>
     <t>external_id</t>
   </si>
@@ -260,6 +260,150 @@
   </si>
   <si>
     <t>Yes, using any TOTP application such as Authy or 1Password. Enable it under Settings, then Security. Save the recovery codes shown at setup: without them, losing the device means contacting support to prove ownership.</t>
+  </si>
+  <si>
+    <t>FAQ-0025</t>
+  </si>
+  <si>
+    <t>How do I change my password without losing my session?</t>
+  </si>
+  <si>
+    <t>Open Settings, then Security, then 'Change password'. Enter the current password once and the new one twice. Other devices stay signed in unless you tick 'Sign out everywhere', which we recommend after a shared login.</t>
+  </si>
+  <si>
+    <t>FAQ-0026</t>
+  </si>
+  <si>
+    <t>Why am I being asked to verify my email again?</t>
+  </si>
+  <si>
+    <t>We re-verify an address after it has been unused for twelve months, or whenever it changes. The link lasts 24 hours. Until it is used, sign-in still works but invoices and reset links are held back.</t>
+  </si>
+  <si>
+    <t>FAQ-0027</t>
+  </si>
+  <si>
+    <t>Can I transfer my account to a colleague?</t>
+  </si>
+  <si>
+    <t>Yes. The current owner opens Settings, then Members, and picks 'Transfer ownership'. The colleague must already be a member and must accept within seven days, after which the transfer expires and nothing changes.</t>
+  </si>
+  <si>
+    <t>FAQ-0028</t>
+  </si>
+  <si>
+    <t>Do you offer refunds on annual plans?</t>
+  </si>
+  <si>
+    <t>We refund an annual plan pro rata within the first 30 days. After that the term runs to its end and renewal stops instead. Refunds go back to the card that paid, and no other method.</t>
+  </si>
+  <si>
+    <t>FAQ-0029</t>
+  </si>
+  <si>
+    <t>How do I update the card on file?</t>
+  </si>
+  <si>
+    <t>Settings, then Billing, then 'Payment method'. Adding a new card replaces the old one immediately; we do not keep a second card as a fallback. A failed renewal retries for five days before the plan is suspended.</t>
+  </si>
+  <si>
+    <t>FAQ-0030</t>
+  </si>
+  <si>
+    <t>Is there a discount for non-profits or education?</t>
+  </si>
+  <si>
+    <t>Registered non-profits and accredited schools get 40% off any plan. Send proof of status from an address on your organisation's domain and we apply it to the next invoice; we do not backdate it.</t>
+  </si>
+  <si>
+    <t>FAQ-0031</t>
+  </si>
+  <si>
+    <t>Can I pick a delivery date?</t>
+  </si>
+  <si>
+    <t>Standard delivery cannot be scheduled. Express delivery lets you choose any working day within the next fortnight at checkout, and the carrier texts a two-hour window on the morning itself.</t>
+  </si>
+  <si>
+    <t>FAQ-0032</t>
+  </si>
+  <si>
+    <t>What happens if nobody is home?</t>
+  </si>
+  <si>
+    <t>The carrier tries twice on consecutive working days, then holds the parcel at the nearest collection point for ten days. After that it comes back to us and we refund the goods but not the original postage.</t>
+  </si>
+  <si>
+    <t>FAQ-0033</t>
+  </si>
+  <si>
+    <t>Do you deliver to PO boxes or parcel lockers?</t>
+  </si>
+  <si>
+    <t>Parcel lockers yes, PO boxes no — our carriers require a signature that a PO box cannot provide. Choose a locker at checkout and you get a one-time code valid for 72 hours.</t>
+  </si>
+  <si>
+    <t>FAQ-0034</t>
+  </si>
+  <si>
+    <t>Can I return an item that was on sale?</t>
+  </si>
+  <si>
+    <t>Sale items can be returned within 14 days rather than the usual 30, and must be unused with tags attached. Clearance items marked 'final sale' cannot be returned unless they arrive faulty.</t>
+  </si>
+  <si>
+    <t>FAQ-0035</t>
+  </si>
+  <si>
+    <t>What if my item arrived damaged?</t>
+  </si>
+  <si>
+    <t>Photograph the damage and the packaging before discarding anything, then start a return and pick 'Arrived damaged'. We ship a replacement the same working day and you keep the damaged item for collection.</t>
+  </si>
+  <si>
+    <t>FAQ-0036</t>
+  </si>
+  <si>
+    <t>How long do I have to change my mind?</t>
+  </si>
+  <si>
+    <t>Thirty days from delivery, counted from the date the carrier records it as delivered rather than from the order date. Opened items are accepted if they are in a condition you would accept yourself.</t>
+  </si>
+  <si>
+    <t>FAQ-0037</t>
+  </si>
+  <si>
+    <t>Do you have rate limits on the API?</t>
+  </si>
+  <si>
+    <t>Sixty requests a minute per token on the free plan and six hundred on paid ones. Exceeding it returns 429 with a Retry-After header. Bursts of double the limit are tolerated for ten seconds.</t>
+  </si>
+  <si>
+    <t>FAQ-0038</t>
+  </si>
+  <si>
+    <t>Can I use webhooks instead of polling?</t>
+  </si>
+  <si>
+    <t>Yes. Register an HTTPS endpoint under Settings, then Developers. We sign every payload with your signing secret and retry a failed delivery six times over an hour before disabling the endpoint.</t>
+  </si>
+  <si>
+    <t>FAQ-0039</t>
+  </si>
+  <si>
+    <t>Is my data encrypted?</t>
+  </si>
+  <si>
+    <t>In transit with TLS 1.3 and at rest with AES-256. Backups are encrypted with a separate key and kept for 35 days. We hold the keys; customer-managed keys are available on the enterprise plan.</t>
+  </si>
+  <si>
+    <t>FAQ-0040</t>
+  </si>
+  <si>
+    <t>Which file formats can I import?</t>
+  </si>
+  <si>
+    <t>CSV and Excel, both up to 50 MB. The first row must be a header, and the columns external_id, question, answer, category and updated_at must all be present. Anything else in the sheet is ignored.</t>
   </si>
 </sst>
 </file>
@@ -321,8 +465,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Frame0" displayName="Frame0" ref="A1:E25" totalsRowShown="0">
-  <autoFilter ref="A1:E25"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Frame0" displayName="Frame0" ref="A1:E41" totalsRowShown="0">
+  <autoFilter ref="A1:E41"/>
   <tableColumns count="5">
     <tableColumn id="1" name="external_id" dataDxfId="0"/>
     <tableColumn id="2" name="question" dataDxfId="0"/>
@@ -619,15 +763,8 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E25"/>
+  <dimension ref="A1:E41"/>
   <sheetFormatPr defaultRowHeight="15"/>
-  <cols>
-    <col min="1" max="1" width="13.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="47.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="211.7109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.85546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.42578125" bestFit="1" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" t="s">
@@ -1052,6 +1189,278 @@
       </c>
       <c r="E25" s="2">
         <v>46101.39583333334</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5">
+      <c r="A26" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="B26" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="C26" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="D26" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="E26" s="2">
+        <v>46222.5</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5">
+      <c r="A27" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="B27" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="C27" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="D27" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="E27" s="2">
+        <v>46222.5</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5">
+      <c r="A28" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="B28" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="C28" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="D28" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="E28" s="2">
+        <v>46222.5</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5">
+      <c r="A29" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="B29" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="C29" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="D29" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="E29" s="2">
+        <v>46222.5</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5">
+      <c r="A30" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="B30" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="C30" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="D30" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="E30" s="2">
+        <v>46222.5</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5">
+      <c r="A31" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="B31" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="C31" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="D31" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="E31" s="2">
+        <v>46222.5</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5">
+      <c r="A32" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="B32" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="C32" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="D32" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="E32" s="2">
+        <v>46222.5</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5">
+      <c r="A33" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="B33" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="C33" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="D33" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="E33" s="2">
+        <v>46222.5</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5">
+      <c r="A34" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="B34" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="C34" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="D34" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="E34" s="2">
+        <v>46222.5</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5">
+      <c r="A35" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="B35" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="C35" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="D35" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="E35" s="2">
+        <v>46222.5</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5">
+      <c r="A36" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="B36" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="C36" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="D36" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="E36" s="2">
+        <v>46222.5</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5">
+      <c r="A37" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="B37" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="C37" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="D37" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="E37" s="2">
+        <v>46222.5</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5">
+      <c r="A38" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="B38" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="C38" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="D38" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="E38" s="2">
+        <v>46222.5</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5">
+      <c r="A39" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="B39" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="C39" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="D39" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="E39" s="2">
+        <v>46222.5</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5">
+      <c r="A40" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="B40" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="C40" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="D40" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="E40" s="2">
+        <v>46222.5</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5">
+      <c r="A41" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="B41" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="C41" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="D41" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="E41" s="2">
+        <v>46222.5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>